<commit_message>
More attempts at video creation
</commit_message>
<xml_diff>
--- a/second-question/metadata/second_question_metadata.xlsx
+++ b/second-question/metadata/second_question_metadata.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release" sheetId="1" r:id="Rf6028c3a11554372"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenes" sheetId="2" r:id="R9fe7a2507aef4178"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rf18a611a4eb84e86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider Profiles" sheetId="4" r:id="R06deb795e52a4e4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rights and Logos" sheetId="5" r:id="R2beb2c98d3c949a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DDEX Crosswalk" sheetId="6" r:id="Raf96d85a4c964abc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="R371f97a9e12f4ae6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release" sheetId="1" r:id="R0f919c61e2ad493e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenes" sheetId="2" r:id="R7ba1a6d67fab4960"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R763e8bc2f9b645df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider Profiles" sheetId="4" r:id="R7437542f7f414041"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rights and Logos" sheetId="5" r:id="R759f68dd69c54486"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DDEX Crosswalk" sheetId="6" r:id="R4fe718480e234bd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rdb461cc5a14e45a9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -43,7 +43,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -60,6 +60,11 @@
         <x:fgColor rgb="FFE5E7EB"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F2937"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -68,7 +73,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="30">
+  <x:cellXfs count="38">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -135,11 +140,59 @@
     <x:xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <xfpb:bag type="Checkbox"/>
+  <xfpb:bag type="XFControls">
+    <xfpb:bagId k="CellControl">0</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplement">
+    <xfpb:bagId k="XFControls">1</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <xfpb:a k="MappedFeaturePropertyBags">
+      <xfpb:bagId>2</xfpb:bagId>
+    </xfpb:a>
+  </xfpb:bag>
+</xfpb:FeaturePropertyBags>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -480,7 +533,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4939561b677547be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53d0e0e98da34785"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -812,7 +865,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2d2150a469340f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea84aa1105d043c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1292,7 +1345,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5578039e0f244441"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96fb4a2f76cd4403"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1336,6 +1389,9 @@
       <x:c r="H1" s="6" t="str">
         <x:v>Notes</x:v>
       </x:c>
+      <x:c r="I1" s="36" t="str">
+        <x:v>Store</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="13" t="str">
@@ -1358,6 +1414,7 @@
       <x:c r="H2" s="13" t="str">
         <x:v>OpenAI Videos API/Sora context visual profile.</x:v>
       </x:c>
+      <x:c r="I2" s="12"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="13" t="str">
@@ -1378,13 +1435,16 @@
         <x:v>uri</x:v>
       </x:c>
       <x:c r="H3" s="13" t="str">
-        <x:v>Gemini Omni Flash Interactions API context visual profile.</x:v>
+        <x:v>Gemini Omni Flash Interactions API context visual profile. URI delivery requires store=true in current API validation.</x:v>
+      </x:c>
+      <x:c r="I3" s="37" t="b">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4a91a2b185c4ed3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6948182a23094d62"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1472,7 +1532,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R250cd7d519d04959"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44da515c622f4bc4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1588,7 +1648,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f7b1916f23a437b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bf09fa5b4124c24"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1690,6 +1750,14 @@
         <x:v>Choose final Creative Commons license, verify source-media reuse rights, and use only official uploaded/downloaded logo assets.</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="12" t="str">
+        <x:v>Gemini Omni URI delivery</x:v>
+      </x:c>
+      <x:c r="B12" s="12" t="str">
+        <x:v>Script now forces store=true when response_format.delivery is uri.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>